<commit_message>
[feat] TrainingData Id를 시설 데이터와 연동
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/TrainingData.xlsx
+++ b/JsonConverter/ExcelFiles/TrainingData.xlsx
@@ -19,102 +19,117 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
-  <x:si>
-    <x:t>TrainingHpPerSecond</x:t>
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+  <x:si>
+    <x:t>cardio_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>standing_strike_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>체력과 경기 스태미너를 기르는 기본 훈련이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스탠딩 타격 훈련</x:t>
+  </x:si>
+  <x:si>
+    <x:t>휴식</x:t>
   </x:si>
   <x:si>
     <x:t>Id</x:t>
   </x:si>
   <x:si>
-    <x:t>휴식</x:t>
-  </x:si>
-  <x:si>
-    <x:t>체력을 올려주는 기본 훈련이다.</x:t>
+    <x:t>standing_strike_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rest_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Training</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ConditionUp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AtkDown</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DefUp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rest</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Time</x:t>
+  </x:si>
+  <x:si>
+    <x:t>AtkUp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HpDown</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DefDown</x:t>
+  </x:si>
+  <x:si>
+    <x:t>float</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HpUp</x:t>
+  </x:si>
+  <x:si>
+    <x:t>더 나은 시설에서 스탠딩 타격 능력을 향상 시키는 훈련이다.</x:t>
   </x:si>
   <x:si>
     <x:t>선수의 컨디션을 회복한다.</x:t>
   </x:si>
   <x:si>
+    <x:t>TrainingType</x:t>
+  </x:si>
+  <x:si>
     <x:t>ConditionDown</x:t>
   </x:si>
   <x:si>
-    <x:t>TrainingType</x:t>
-  </x:si>
-  <x:si>
-    <x:t>training_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Training</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ConditionUp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>training_02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>training_00</x:t>
-  </x:si>
-  <x:si>
-    <x:t>training_03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HpUp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>방어력훈련</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DefDown</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DefUp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>체력훈련</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AtkUp</x:t>
-  </x:si>
-  <x:si>
-    <x:t>공격력훈련</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>float</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Rest</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>AtkDown</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HpDown</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Time</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선수의 펀치력을 향상시키는 훈련이다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>선수의 방어능력을 향상시키는 훈련이다.</x:t>
+    <x:t>standing_def_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선수의 컨디션을 조금 더 회복한다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>카디오 훈련</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선수의 스탠딩 방어 능력을 향상시키는 훈련이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개선된 휴식</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rest_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>스탠딩 방어 훈련</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개선된 스탠딩 타격 훈련</x:t>
+  </x:si>
+  <x:si>
+    <x:t>선수의 스탠딩 타격 능력을 향상시키는 훈련이다.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -885,180 +900,171 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:N35"/>
+  <x:dimension ref="A1:M35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="25.4296875" style="1" customWidth="1"/>
     <x:col min="2" max="2" width="19.54296875" style="1" customWidth="1"/>
-    <x:col min="3" max="3" width="50.7265625" style="1" customWidth="1"/>
-    <x:col min="4" max="6" width="20.26953125" style="1" customWidth="1"/>
-    <x:col min="7" max="7" width="30.54296875" style="1" customWidth="1"/>
-    <x:col min="8" max="8" width="26.54296875" style="1" customWidth="1"/>
-    <x:col min="9" max="9" width="20" style="1" customWidth="1"/>
-    <x:col min="10" max="12" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
-    <x:col min="13" max="13" width="15.71484375" style="1" customWidth="1"/>
-    <x:col min="14" max="14" width="17.4296875" style="1" customWidth="1"/>
-    <x:col min="15" max="16384" width="12.54296875" style="1"/>
+    <x:col min="3" max="3" width="41.5703125" style="1" customWidth="1"/>
+    <x:col min="4" max="5" width="20.26953125" style="1" customWidth="1"/>
+    <x:col min="6" max="6" width="30.54296875" style="1" customWidth="1"/>
+    <x:col min="7" max="7" width="26.54296875" style="1" customWidth="1"/>
+    <x:col min="8" max="8" width="20" style="1" customWidth="1"/>
+    <x:col min="9" max="11" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
+    <x:col min="12" max="12" width="15.71484375" style="1" customWidth="1"/>
+    <x:col min="13" max="13" width="17.4296875" style="1" customWidth="1"/>
+    <x:col min="14" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:13" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="I2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="J2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M2" s="1" t="s">
+        <x:v>21</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:13" s="7" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C3" s="7" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D3" s="7" t="s">
         <x:v>26</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:14" ht="13.199999999999999">
-      <x:c r="A2" s="1" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
+      <x:c r="E3" s="7" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="F3" s="7" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="H2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="I2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="J2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="K2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="M2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="N2" s="1" t="s">
-        <x:v>23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:14" s="7" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="2" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
+      <x:c r="G3" s="7" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H3" s="7" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J3" s="7" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="K3" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="L3" s="7" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="M3" s="7" t="s">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="A4" s="3" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="D3" s="7" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="E3" s="7" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="F3" s="7" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G3" s="7" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="H3" s="7" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="I3" s="7" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="J3" s="7" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="K3" s="7" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="L3" s="7" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="M3" s="7" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="N3" s="7" t="s">
-        <x:v>5</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:14" ht="15.75" customHeight="1">
-      <x:c r="A4" s="3" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B4" s="3" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="s">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="D4" s="1" t="s">
-        <x:v>24</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E4" s="1">
         <x:v>10</x:v>
       </x:c>
       <x:c r="F4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" s="4">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L4" s="1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="M4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="A5" s="3" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C5" s="1" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E5" s="1">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H4" s="4">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M4" s="1">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="N4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:14" ht="15.75" customHeight="1">
-      <x:c r="A5" s="3" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B5" s="3" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="C5" s="3" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D5" s="1" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E5" s="1">
-        <x:v>20</x:v>
-      </x:c>
       <x:c r="F5" s="1">
-        <x:v>-5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G5" s="1">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H5" s="1">
         <x:v>0</x:v>
@@ -1073,33 +1079,30 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L5" s="1">
-        <x:v>0</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="M5" s="1">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="N5" s="1">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:14" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="6" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="C6" s="5" t="s">
         <x:v>30</x:v>
       </x:c>
+      <x:c r="C6" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E6" s="1">
         <x:v>20</x:v>
       </x:c>
       <x:c r="F6" s="1">
-        <x:v>-4</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G6" s="1">
         <x:v>0</x:v>
@@ -1108,49 +1111,46 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="I6" s="1">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J6" s="1">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K6" s="1">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="L6" s="1">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N6" s="1">
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" spans="1:14" ht="15.75" customHeight="1">
+    <x:row r="7" spans="1:13" ht="15.75" customHeight="1">
       <x:c r="A7" s="5" t="s">
-        <x:v>13</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="C7" s="5" t="s">
-        <x:v>31</x:v>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C7" s="1" t="s">
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E7" s="1">
         <x:v>20</x:v>
       </x:c>
       <x:c r="F7" s="1">
-        <x:v>-4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G7" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H7" s="1">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H7" s="1">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="I7" s="1">
         <x:v>0</x:v>
       </x:c>
@@ -1158,141 +1158,188 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="K7" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L7" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M7" s="1">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="A8" s="5" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C8" s="1" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E8" s="1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F8" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G8" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H8" s="1">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="I8" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J8" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="K8" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L8" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M8" s="1">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:13" ht="15.75" customHeight="1">
+      <x:c r="A9" s="5" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="C9" s="1" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E9" s="1">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F9" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H9" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I9" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J9" s="1">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="L7" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M7" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N7" s="1">
+      <x:c r="K9" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L9" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M9" s="1">
         <x:v>10</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A8" s="5"/>
-      <x:c r="B8" s="5"/>
-      <x:c r="C8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A9" s="5"/>
-      <x:c r="B9" s="5"/>
-      <x:c r="C9" s="5"/>
     </x:row>
     <x:row r="10" ht="15.75" customHeight="1"/>
     <x:row r="11" ht="15.75" customHeight="1"/>
-    <x:row r="12" spans="1:3" ht="15.75" customHeight="1">
+    <x:row r="12" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A12" s="6"/>
       <x:c r="B12" s="6"/>
-      <x:c r="C12" s="6"/>
-    </x:row>
-    <x:row r="13" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="13" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A13" s="3"/>
       <x:c r="B13" s="3"/>
-      <x:c r="C13" s="3"/>
     </x:row>
     <x:row r="14" ht="15.75" customHeight="1"/>
     <x:row r="15" ht="15.75" customHeight="1"/>
-    <x:row r="16" spans="1:3" ht="15.75" customHeight="1">
+    <x:row r="16" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A16" s="5"/>
       <x:c r="B16" s="5"/>
-      <x:c r="C16" s="5"/>
-    </x:row>
-    <x:row r="17" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="17" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A17" s="5"/>
       <x:c r="B17" s="5"/>
-      <x:c r="C17" s="5"/>
-    </x:row>
-    <x:row r="18" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="18" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A18" s="5"/>
       <x:c r="B18" s="5"/>
-      <x:c r="C18" s="5"/>
-    </x:row>
-    <x:row r="19" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="19" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A19" s="5"/>
       <x:c r="B19" s="5"/>
-      <x:c r="C19" s="5"/>
-    </x:row>
-    <x:row r="20" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="20" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A20" s="5"/>
       <x:c r="B20" s="5"/>
-      <x:c r="C20" s="5"/>
-    </x:row>
-    <x:row r="21" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="21" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A21" s="5"/>
       <x:c r="B21" s="5"/>
-      <x:c r="C21" s="5"/>
-    </x:row>
-    <x:row r="22" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="22" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A22" s="5"/>
       <x:c r="B22" s="5"/>
-      <x:c r="C22" s="5"/>
-    </x:row>
-    <x:row r="23" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="23" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A23" s="5"/>
       <x:c r="B23" s="5"/>
-      <x:c r="C23" s="5"/>
-    </x:row>
-    <x:row r="24" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="24" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A24" s="5"/>
       <x:c r="B24" s="5"/>
-      <x:c r="C24" s="5"/>
-    </x:row>
-    <x:row r="25" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="25" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A25" s="5"/>
       <x:c r="B25" s="5"/>
-      <x:c r="C25" s="5"/>
-    </x:row>
-    <x:row r="26" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="26" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A26" s="6"/>
       <x:c r="B26" s="6"/>
-      <x:c r="C26" s="6"/>
-    </x:row>
-    <x:row r="27" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="27" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A27" s="6"/>
       <x:c r="B27" s="6"/>
-      <x:c r="C27" s="6"/>
-    </x:row>
-    <x:row r="28" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="28" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A28" s="6"/>
       <x:c r="B28" s="6"/>
-      <x:c r="C28" s="6"/>
-    </x:row>
-    <x:row r="29" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="29" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A29" s="6"/>
       <x:c r="B29" s="6"/>
-      <x:c r="C29" s="6"/>
-    </x:row>
-    <x:row r="30" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="30" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A30" s="6"/>
       <x:c r="B30" s="6"/>
-      <x:c r="C30" s="6"/>
-    </x:row>
-    <x:row r="31" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="31" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A31" s="6"/>
       <x:c r="B31" s="6"/>
-      <x:c r="C31" s="6"/>
-    </x:row>
-    <x:row r="32" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="32" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A32" s="3"/>
       <x:c r="B32" s="3"/>
-      <x:c r="C32" s="3"/>
-    </x:row>
-    <x:row r="33" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="33" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A33" s="3"/>
       <x:c r="B33" s="3"/>
-      <x:c r="C33" s="3"/>
-    </x:row>
-    <x:row r="34" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="34" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A34" s="3"/>
       <x:c r="B34" s="3"/>
-      <x:c r="C34" s="3"/>
-    </x:row>
-    <x:row r="35" spans="1:3" ht="15.75" customHeight="1">
+    </x:row>
+    <x:row r="35" spans="1:2" ht="15.75" customHeight="1">
       <x:c r="A35" s="3"/>
       <x:c r="B35" s="3"/>
-      <x:c r="C35" s="3"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1"/>
     <x:row r="37" ht="15.75" customHeight="1"/>

</xml_diff>